<commit_message>
Update scripts and add inter rater statistics with Cohen's kappa.
</commit_message>
<xml_diff>
--- a/data/query_results/prisma_screening_process.xlsx
+++ b/data/query_results/prisma_screening_process.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mariambzd\repos\bibMining\data\query_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A97467-9C87-4025-B064-815FC575AC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{316FB2C8-322B-4E4A-B64C-762378B683A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,9 +23,9 @@
     <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Corpus!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Corpus!$A$1:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Eligibility!$A$1:$M$67</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Inclusion!$A$1:$J$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Inclusion!$A$1:$J$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Screening!$A$1:$M$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2052" uniqueCount="920">
   <si>
     <t>Title</t>
   </si>
@@ -2775,15 +2775,6 @@
     <t>Indonesia</t>
   </si>
   <si>
-    <t>Social innovation ecological crises and creating mining host community resilience in Southern Africa</t>
-  </si>
-  <si>
-    <t>Chipangamate; Nwaila</t>
-  </si>
-  <si>
-    <t>Social innovation;Community resilience;Monitoring;Evaluation;Social Learning;Climate change;Biodiversity loss;Social innovation assessment</t>
-  </si>
-  <si>
     <t>Sustainable Water-Related Hazards Assessment in Open Pit-to-Underground Mining Transitions: An IDRR and MCDM Approach at Sijiaying Iron Mine, China</t>
   </si>
   <si>
@@ -2812,6 +2803,9 @@
   </si>
   <si>
     <t>Tri-AHP; coal mine; rainstorm; well flooding; vulnerability; risk assessment; environmental sustainability</t>
+  </si>
+  <si>
+    <t>not_case_study</t>
   </si>
 </sst>
 </file>
@@ -12686,7 +12680,7 @@
         <v>out_of_scope</v>
       </c>
     </row>
-    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>75</v>
       </c>
@@ -12717,9 +12711,11 @@
       <c r="K38" t="s">
         <v>437</v>
       </c>
-      <c r="L38" t="str">
-        <f>VLOOKUP(B38,[2]Hoja1!A:E,4,FALSE)</f>
-        <v>included</v>
+      <c r="L38" t="s">
+        <v>778</v>
+      </c>
+      <c r="M38" t="s">
+        <v>919</v>
       </c>
     </row>
     <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.3">
@@ -13921,7 +13917,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{121CF889-D7FF-44E7-AA83-BC59A31FB3ED}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -14144,10 +14140,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>432</v>
+        <v>488</v>
       </c>
       <c r="B8" t="s">
-        <v>433</v>
+        <v>489</v>
       </c>
       <c r="C8">
         <v>2025</v>
@@ -14156,27 +14152,30 @@
         <v>170</v>
       </c>
       <c r="E8" t="s">
-        <v>434</v>
+        <v>490</v>
       </c>
       <c r="F8" t="s">
-        <v>435</v>
+        <v>491</v>
       </c>
       <c r="G8" t="s">
-        <v>436</v>
+        <v>492</v>
+      </c>
+      <c r="H8" t="s">
+        <v>493</v>
       </c>
       <c r="I8" t="s">
         <v>17</v>
       </c>
       <c r="J8" t="s">
-        <v>437</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>488</v>
+        <v>605</v>
       </c>
       <c r="B9" t="s">
-        <v>489</v>
+        <v>606</v>
       </c>
       <c r="C9">
         <v>2025</v>
@@ -14185,16 +14184,16 @@
         <v>170</v>
       </c>
       <c r="E9" t="s">
-        <v>490</v>
+        <v>607</v>
       </c>
       <c r="F9" t="s">
-        <v>491</v>
+        <v>608</v>
       </c>
       <c r="G9" t="s">
-        <v>492</v>
+        <v>609</v>
       </c>
       <c r="H9" t="s">
-        <v>493</v>
+        <v>610</v>
       </c>
       <c r="I9" t="s">
         <v>17</v>
@@ -14205,10 +14204,10 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>605</v>
+        <v>660</v>
       </c>
       <c r="B10" t="s">
-        <v>606</v>
+        <v>661</v>
       </c>
       <c r="C10">
         <v>2025</v>
@@ -14217,16 +14216,13 @@
         <v>170</v>
       </c>
       <c r="E10" t="s">
-        <v>607</v>
+        <v>662</v>
       </c>
       <c r="F10" t="s">
-        <v>608</v>
+        <v>663</v>
       </c>
       <c r="G10" t="s">
-        <v>609</v>
-      </c>
-      <c r="H10" t="s">
-        <v>610</v>
+        <v>664</v>
       </c>
       <c r="I10" t="s">
         <v>17</v>
@@ -14237,25 +14233,25 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>660</v>
+        <v>706</v>
       </c>
       <c r="B11" t="s">
-        <v>661</v>
+        <v>707</v>
       </c>
       <c r="C11">
-        <v>2025</v>
+        <v>2023</v>
       </c>
       <c r="D11" t="s">
         <v>170</v>
       </c>
       <c r="E11" t="s">
-        <v>662</v>
+        <v>708</v>
       </c>
       <c r="F11" t="s">
-        <v>663</v>
+        <v>709</v>
       </c>
       <c r="G11" t="s">
-        <v>664</v>
+        <v>710</v>
       </c>
       <c r="I11" t="s">
         <v>17</v>
@@ -14266,25 +14262,28 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>706</v>
+        <v>713</v>
       </c>
       <c r="B12" t="s">
-        <v>707</v>
+        <v>612</v>
       </c>
       <c r="C12">
-        <v>2023</v>
+        <v>2021</v>
       </c>
       <c r="D12" t="s">
         <v>170</v>
       </c>
       <c r="E12" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="F12" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="G12" t="s">
-        <v>710</v>
+        <v>716</v>
+      </c>
+      <c r="H12" t="s">
+        <v>717</v>
       </c>
       <c r="I12" t="s">
         <v>17</v>
@@ -14293,47 +14292,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>713</v>
-      </c>
-      <c r="B13" t="s">
-        <v>612</v>
-      </c>
-      <c r="C13">
-        <v>2021</v>
-      </c>
-      <c r="D13" t="s">
-        <v>170</v>
-      </c>
-      <c r="E13" t="s">
-        <v>714</v>
-      </c>
-      <c r="F13" t="s">
-        <v>715</v>
-      </c>
-      <c r="G13" t="s">
-        <v>716</v>
-      </c>
-      <c r="H13" t="s">
-        <v>717</v>
-      </c>
-      <c r="I13" t="s">
-        <v>17</v>
-      </c>
-      <c r="J13" t="s">
-        <v>18</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J13" xr:uid="{121CF889-D7FF-44E7-AA83-BC59A31FB3ED}"/>
+  <autoFilter ref="A1:J12" xr:uid="{121CF889-D7FF-44E7-AA83-BC59A31FB3ED}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A4D3F1-AC14-4FBF-9F06-5A47518AF103}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" customWidth="1"/>
@@ -15059,25 +15026,25 @@
         <v>909</v>
       </c>
       <c r="B27" t="s">
-        <v>910</v>
+        <v>788</v>
       </c>
       <c r="C27">
         <v>2025</v>
       </c>
       <c r="D27" t="s">
-        <v>807</v>
+        <v>910</v>
       </c>
       <c r="E27" t="s">
         <v>790</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G27" t="s">
-        <v>797</v>
+        <v>791</v>
       </c>
       <c r="H27" t="s">
-        <v>792</v>
+        <v>894</v>
       </c>
       <c r="I27" t="s">
         <v>911</v>
@@ -15088,28 +15055,22 @@
         <v>912</v>
       </c>
       <c r="B28" t="s">
-        <v>788</v>
+        <v>913</v>
       </c>
       <c r="C28">
         <v>2025</v>
       </c>
       <c r="D28" t="s">
-        <v>913</v>
+        <v>914</v>
       </c>
       <c r="E28" t="s">
         <v>790</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G28" t="s">
-        <v>791</v>
-      </c>
-      <c r="H28" t="s">
-        <v>894</v>
-      </c>
-      <c r="I28" t="s">
-        <v>914</v>
+        <v>818</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -15120,52 +15081,29 @@
         <v>916</v>
       </c>
       <c r="C29">
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="D29" t="s">
-        <v>917</v>
+        <v>855</v>
       </c>
       <c r="E29" t="s">
         <v>790</v>
       </c>
       <c r="F29">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G29" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+        <v>791</v>
+      </c>
+      <c r="H29" t="s">
+        <v>917</v>
+      </c>
+      <c r="I29" t="s">
         <v>918</v>
       </c>
-      <c r="B30" t="s">
-        <v>919</v>
-      </c>
-      <c r="C30">
-        <v>2022</v>
-      </c>
-      <c r="D30" t="s">
-        <v>855</v>
-      </c>
-      <c r="E30" t="s">
-        <v>790</v>
-      </c>
-      <c r="F30">
-        <v>5</v>
-      </c>
-      <c r="G30" t="s">
-        <v>791</v>
-      </c>
-      <c r="H30" t="s">
-        <v>920</v>
-      </c>
-      <c r="I30" t="s">
-        <v>921</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I30" xr:uid="{63A4D3F1-AC14-4FBF-9F06-5A47518AF103}"/>
+  <autoFilter ref="A1:I29" xr:uid="{63A4D3F1-AC14-4FBF-9F06-5A47518AF103}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>